<commit_message>
Update INFOR Buyers List Template conditional formatting
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Buyers List Template.xlsx
+++ b/infor-workflows/templates/INFOR Buyers List Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude Access Folder/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude - INFOR/infor-workflows/infor-workflows/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6757E3D-B2F3-46E9-ACCD-D08BA7BD5904}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6CE1705-7D95-4A90-B156-E0277A9A2B3D}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -178,8 +178,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="166" formatCode="#,##0_);\(#,##0\);&quot;--&quot;"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\);&quot;--&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0_);\(#,##0\);&quot;--&quot;"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\);&quot;--&quot;"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -330,7 +330,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -352,42 +352,25 @@
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -396,19 +379,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -416,6 +396,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -426,21 +409,14 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
-        <color theme="9"/>
+        <color rgb="FF00B050"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor rgb="FFCCFFCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -464,7 +440,7 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor rgb="FFFFCCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -479,11 +455,11 @@
       <font>
         <b/>
         <i val="0"/>
-        <color theme="9"/>
+        <color rgb="FF00B050"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor rgb="FFCCFFCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -507,7 +483,14 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -515,6 +498,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCCFFCC"/>
+      <color rgb="FFFFCCCC"/>
       <color rgb="FFF3F6CC"/>
     </mruColors>
   </colors>
@@ -869,73 +854,73 @@
       <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
     </row>
     <row r="5" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
     </row>
     <row r="6" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
     </row>
     <row r="7" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
     </row>
     <row r="8" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
     </row>
     <row r="9" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
     </row>
     <row r="10" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
     </row>
     <row r="11" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
     </row>
     <row r="12" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -946,78 +931,78 @@
       <c r="D13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="25" t="s">
+      <c r="F13" s="18" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="26"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="19"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="17">
         <f>+'Strategic Buyers'!$H$25</f>
         <v>0</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="17">
         <f>+'Strategic Buyers'!$H$26</f>
         <v>0</v>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="17">
         <f>+'Strategic Buyers'!$H$27</f>
         <v>0</v>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="20">
         <f>SUM(C15:E15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="17">
         <f>+'Financial Buyers'!$I$25</f>
         <v>0</v>
       </c>
-      <c r="D16" s="24">
+      <c r="D16" s="17">
         <f>+'Financial Buyers'!$I$26</f>
         <v>0</v>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="17">
         <f>+'Financial Buyers'!$I$27</f>
         <v>0</v>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="20">
         <f>SUM(C16:E16)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="30">
+      <c r="C17" s="22">
         <f>SUM(C15:C16)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="30">
+      <c r="D17" s="22">
         <f t="shared" ref="D17:F17" si="0">SUM(D15:D16)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="30">
+      <c r="E17" s="22">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F17" s="31">
+      <c r="F17" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1039,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16A72140-9B00-4D9F-A775-351377C5BFAB}">
-  <dimension ref="B2:H28"/>
+  <dimension ref="B2:H27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
@@ -1052,38 +1037,38 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="32" t="s">
+      <c r="F2" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="32" t="s">
+      <c r="E3" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="F3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="G3" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="24" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1092,211 +1077,200 @@
       <c r="B5" s="8"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="18"/>
+      <c r="E5" s="15"/>
       <c r="F5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B6" s="8"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
-      <c r="E6" s="19"/>
-      <c r="H6" s="2"/>
+      <c r="E6" s="16"/>
+      <c r="H6" s="26"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="8"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="19"/>
-      <c r="H7" s="2"/>
+      <c r="E7" s="16"/>
+      <c r="H7" s="26"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="8"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
-      <c r="E8" s="19"/>
-      <c r="H8" s="2"/>
+      <c r="E8" s="16"/>
+      <c r="H8" s="26"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
-      <c r="E9" s="19"/>
-      <c r="H9" s="2"/>
+      <c r="E9" s="16"/>
+      <c r="H9" s="26"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="8"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
-      <c r="E10" s="19"/>
-      <c r="H10" s="2"/>
+      <c r="E10" s="16"/>
+      <c r="H10" s="26"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="8"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
-      <c r="E11" s="19"/>
-      <c r="H11" s="2"/>
+      <c r="E11" s="16"/>
+      <c r="H11" s="26"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="8"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="19"/>
-      <c r="H12" s="2"/>
+      <c r="E12" s="16"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" s="8"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="19"/>
-      <c r="H13" s="2"/>
+      <c r="E13" s="16"/>
+      <c r="H13" s="26"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14" s="8"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="19"/>
-      <c r="H14" s="2"/>
+      <c r="E14" s="16"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15" s="8"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="19"/>
-      <c r="H15" s="2"/>
+      <c r="E15" s="16"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16" s="8"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="19"/>
-      <c r="H16" s="2"/>
+      <c r="E16" s="16"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17" s="8"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="19"/>
-      <c r="H17" s="2"/>
+      <c r="E17" s="16"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="8"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="19"/>
-      <c r="H18" s="2"/>
+      <c r="E18" s="16"/>
+      <c r="H18" s="26"/>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="8"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="19"/>
-      <c r="H19" s="2"/>
+      <c r="E19" s="16"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="8"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="19"/>
-      <c r="H20" s="2"/>
+      <c r="E20" s="16"/>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21" s="8"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="19"/>
-      <c r="H21" s="2"/>
+      <c r="E21" s="16"/>
+      <c r="H21" s="26"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B22" s="8"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="19"/>
-      <c r="H22" s="2"/>
+      <c r="E22" s="16"/>
+      <c r="H22" s="26"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B23" s="8"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
-      <c r="E23" s="19"/>
-      <c r="H23" s="2"/>
+      <c r="E23" s="16"/>
+      <c r="H23" s="26"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B24" s="9"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="11"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="16"/>
+      <c r="H24" s="26"/>
     </row>
     <row r="25" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="13">
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="10">
         <f>COUNTIF($H$5:$H$24,"A")</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="15">
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="12">
         <f>COUNTIF($H$5:$H$24,"B")</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="17">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="14">
         <f>COUNTIF($H$5:$H$24,"C")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-    </row>
   </sheetData>
+  <conditionalFormatting sqref="B5:G24">
+    <cfRule type="expression" dxfId="7" priority="4">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H5:H24">
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>"A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:H24">
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1305,7 +1279,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{867F1A7A-94AB-4F33-BEE5-43785A42D7B2}">
-  <dimension ref="B2:I28"/>
+  <dimension ref="B2:I27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
@@ -1318,46 +1292,46 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="32" t="s">
+      <c r="E2" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="32" t="s">
+      <c r="F2" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="32" t="s">
+      <c r="G2" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="32" t="s">
+      <c r="D3" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="32" t="s">
+      <c r="E3" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="F3" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="32" t="s">
+      <c r="G3" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="33" t="s">
+      <c r="H3" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="I3" s="32" t="s">
+      <c r="I3" s="24" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1365,236 +1339,224 @@
     <row r="5" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B5" s="8"/>
       <c r="C5" s="2"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
       <c r="G5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="I5" s="26"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B6" s="8"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B7" s="8"/>
       <c r="C7" s="2"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B8" s="8"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="19"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B10" s="8"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B11" s="8"/>
       <c r="C11" s="2"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B12" s="8"/>
       <c r="C12" s="2"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B13" s="8"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
       <c r="I13" s="2"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B14" s="8"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
       <c r="I14" s="2"/>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B15" s="8"/>
       <c r="C15" s="2"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
       <c r="I15" s="2"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B16" s="8"/>
       <c r="C16" s="2"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
       <c r="I16" s="2"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B17" s="8"/>
       <c r="C17" s="2"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
       <c r="I17" s="2"/>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B18" s="8"/>
       <c r="C18" s="2"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
       <c r="I18" s="2"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B19" s="8"/>
       <c r="C19" s="2"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
       <c r="I19" s="2"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B20" s="8"/>
       <c r="C20" s="2"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
       <c r="I20" s="2"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B21" s="8"/>
       <c r="C21" s="2"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
       <c r="I21" s="2"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B22" s="8"/>
       <c r="C22" s="2"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
       <c r="I22" s="2"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B23" s="8"/>
       <c r="C23" s="2"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
       <c r="I23" s="2"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B24" s="9"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="11"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="I24" s="2"/>
     </row>
     <row r="25" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="13">
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="10">
         <f>COUNTIF($I$5:$I$24,"A")</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15">
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="12">
         <f>COUNTIF($I$5:$I$24,"B")</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="16" t="s">
+      <c r="B27" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="17">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="14">
         <f>COUNTIF($I$5:$I$24,"C")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-    </row>
   </sheetData>
+  <conditionalFormatting sqref="B5:H24">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>ISEVEN(ROW())</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I5:I24">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
       <formula>"A"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5:I24">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>ISEVEN(ROW())</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Expand buyerslist-infor rationale column to professional IB prose
The Buyers List template now uses taller data rows with wrap_text on the
Rationale columns, so rationales are written as 1–2 full IB-style
sentences (~150–350 chars) instead of cramped ≤50-char shorthand. The
Financial Buyers column previously labelled "Portfolio Overlap / Add-On
Target" is renamed to "Rationale" to match the Strategic sheet.

SKILL.md adds a Rationale Writing Guidelines section with voice/register
rules, a content-by-buyer-type table, and strong vs. weak examples.

Adds Step 7b, which deletes unused rows between the last populated buyer
and the Tier totals on each buyer sheet, and rewrites the COUNTIF and
Summary cross-sheet references at their new row positions so the
Target Overview tier totals stay correct regardless of how many buyers
are written.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Buyers List Template.xlsx
+++ b/infor-workflows/templates/INFOR Buyers List Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude - INFOR/infor-workflows/infor-workflows/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6CE1705-7D95-4A90-B156-E0277A9A2B3D}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90E98805-2EDB-4877-A873-C05257454523}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>Company</t>
   </si>
@@ -165,9 +165,6 @@
   </si>
   <si>
     <t>Avg. Deal</t>
-  </si>
-  <si>
-    <t>Portfolio Overlap / Add-On Target</t>
   </si>
   <si>
     <t>Size (C$B)</t>
@@ -330,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -402,6 +399,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1073,103 +1073,117 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="15"/>
       <c r="F5" s="2"/>
+      <c r="G5" s="28"/>
       <c r="H5" s="26"/>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="8"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="16"/>
+      <c r="G6" s="28"/>
       <c r="H6" s="26"/>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="16"/>
+      <c r="G7" s="28"/>
       <c r="H7" s="26"/>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="16"/>
+      <c r="G8" s="28"/>
       <c r="H8" s="26"/>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="16"/>
+      <c r="G9" s="28"/>
       <c r="H9" s="26"/>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="8"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="16"/>
+      <c r="G10" s="28"/>
       <c r="H10" s="26"/>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="8"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="16"/>
+      <c r="G11" s="28"/>
       <c r="H11" s="26"/>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="8"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="16"/>
+      <c r="G12" s="28"/>
       <c r="H12" s="26"/>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="8"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="16"/>
+      <c r="G13" s="28"/>
       <c r="H13" s="26"/>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="8"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="16"/>
+      <c r="G14" s="28"/>
       <c r="H14" s="26"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="8"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="16"/>
+      <c r="G15" s="28"/>
       <c r="H15" s="26"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="8"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="16"/>
+      <c r="G16" s="28"/>
       <c r="H16" s="26"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="8"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="16"/>
+      <c r="G17" s="28"/>
       <c r="H17" s="26"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="8"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="16"/>
+      <c r="G18" s="28"/>
       <c r="H18" s="26"/>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.3">
@@ -1177,41 +1191,47 @@
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="16"/>
+      <c r="G19" s="28"/>
       <c r="H19" s="26"/>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="8"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="16"/>
+      <c r="G20" s="28"/>
       <c r="H20" s="26"/>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="8"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="16"/>
+      <c r="G21" s="28"/>
       <c r="H21" s="26"/>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="8"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="16"/>
+      <c r="G22" s="28"/>
       <c r="H22" s="26"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="8"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="16"/>
+      <c r="G23" s="28"/>
       <c r="H23" s="26"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="8"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="16"/>
+      <c r="G24" s="28"/>
       <c r="H24" s="26"/>
     </row>
     <row r="25" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1317,7 +1337,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E3" s="24" t="s">
         <v>28</v>
@@ -1329,172 +1349,192 @@
         <v>29</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="I3" s="24" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8"/>
       <c r="C5" s="2"/>
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
       <c r="G5" s="2"/>
+      <c r="H5" s="28"/>
       <c r="I5" s="26"/>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="8"/>
       <c r="C6" s="2"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
+      <c r="H6" s="28"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8"/>
       <c r="C7" s="2"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
+      <c r="H7" s="28"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="8"/>
       <c r="C8" s="2"/>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
+      <c r="H8" s="28"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="2"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
+      <c r="H9" s="28"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="8"/>
       <c r="C10" s="2"/>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
+      <c r="H10" s="28"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="8"/>
       <c r="C11" s="2"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
+      <c r="H11" s="28"/>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="8"/>
       <c r="C12" s="2"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
+      <c r="H12" s="28"/>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="8"/>
       <c r="C13" s="2"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
+      <c r="H13" s="28"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="8"/>
       <c r="C14" s="2"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
+      <c r="H14" s="28"/>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="8"/>
       <c r="C15" s="2"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
+      <c r="H15" s="28"/>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="8"/>
       <c r="C16" s="2"/>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
       <c r="F16" s="16"/>
+      <c r="H16" s="28"/>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="8"/>
       <c r="C17" s="2"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
+      <c r="H17" s="28"/>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="8"/>
       <c r="C18" s="2"/>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
       <c r="F18" s="16"/>
+      <c r="H18" s="28"/>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="8"/>
       <c r="C19" s="2"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
+      <c r="H19" s="28"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="8"/>
       <c r="C20" s="2"/>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
+      <c r="H20" s="28"/>
       <c r="I20" s="2"/>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="8"/>
       <c r="C21" s="2"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
+      <c r="H21" s="28"/>
       <c r="I21" s="2"/>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="8"/>
       <c r="C22" s="2"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16"/>
       <c r="F22" s="16"/>
+      <c r="H22" s="28"/>
       <c r="I22" s="2"/>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="8"/>
       <c r="C23" s="2"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
+      <c r="H23" s="28"/>
       <c r="I23" s="2"/>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="8"/>
       <c r="C24" s="2"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
+      <c r="H24" s="28"/>
       <c r="I24" s="2"/>
     </row>
     <row r="25" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update INFOR Buyers List Template to fix conditional formatting
Replaces the buyerslist-infor template with a corrected version that
resolves conditional formatting issues introduced in the prior update.
No cell references changed.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Buyers List Template.xlsx
+++ b/infor-workflows/templates/INFOR Buyers List Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude - INFOR/infor-workflows/infor-workflows/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude Access Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6CE1705-7D95-4A90-B156-E0277A9A2B3D}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66AD0C38-56CC-485A-ABB5-17C52B174AF8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
   <si>
     <t>Company</t>
   </si>
@@ -165,9 +165,6 @@
   </si>
   <si>
     <t>Avg. Deal</t>
-  </si>
-  <si>
-    <t>Portfolio Overlap / Add-On Target</t>
   </si>
   <si>
     <t>Size (C$B)</t>
@@ -330,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -397,17 +394,37 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="7">
     <dxf>
       <font>
         <b/>
@@ -441,13 +458,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFCCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1073,146 +1083,176 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="15"/>
       <c r="F5" s="2"/>
-      <c r="H5" s="26"/>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B6" s="8"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="16"/>
-      <c r="H6" s="26"/>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G5" s="26"/>
+      <c r="H5" s="28"/>
+    </row>
+    <row r="6" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="29"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="35"/>
+    </row>
+    <row r="7" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="16"/>
-      <c r="H7" s="26"/>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B8" s="8"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="16"/>
-      <c r="H8" s="26"/>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G7" s="26"/>
+      <c r="H7" s="28"/>
+    </row>
+    <row r="8" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="29"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="35"/>
+    </row>
+    <row r="9" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="16"/>
-      <c r="H9" s="26"/>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="8"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="16"/>
-      <c r="H10" s="26"/>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G9" s="26"/>
+      <c r="H9" s="28"/>
+    </row>
+    <row r="10" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="29"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="35"/>
+    </row>
+    <row r="11" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="8"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="16"/>
-      <c r="H11" s="26"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="8"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="16"/>
-      <c r="H12" s="26"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G11" s="26"/>
+      <c r="H11" s="28"/>
+    </row>
+    <row r="12" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="29"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="35"/>
+    </row>
+    <row r="13" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="8"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="16"/>
-      <c r="H13" s="26"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="8"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="16"/>
-      <c r="H14" s="26"/>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G13" s="26"/>
+      <c r="H13" s="28"/>
+    </row>
+    <row r="14" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="29"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="35"/>
+    </row>
+    <row r="15" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="8"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="16"/>
-      <c r="H15" s="26"/>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="8"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="16"/>
-      <c r="H16" s="26"/>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G15" s="26"/>
+      <c r="H15" s="28"/>
+    </row>
+    <row r="16" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="29"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="35"/>
+    </row>
+    <row r="17" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="8"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="16"/>
-      <c r="H17" s="26"/>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B18" s="8"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="16"/>
-      <c r="H18" s="26"/>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G17" s="26"/>
+      <c r="H17" s="28"/>
+    </row>
+    <row r="18" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="35"/>
+    </row>
+    <row r="19" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="8"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="16"/>
-      <c r="H19" s="26"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B20" s="8"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="16"/>
-      <c r="H20" s="26"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G19" s="26"/>
+      <c r="H19" s="28"/>
+    </row>
+    <row r="20" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="29"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="35"/>
+    </row>
+    <row r="21" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="8"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="16"/>
-      <c r="H21" s="26"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="8"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="16"/>
-      <c r="H22" s="26"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="G21" s="26"/>
+      <c r="H21" s="28"/>
+    </row>
+    <row r="22" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="29"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="33"/>
+      <c r="H22" s="35"/>
+    </row>
+    <row r="23" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="8"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="16"/>
-      <c r="H23" s="26"/>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B24" s="8"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="16"/>
-      <c r="H24" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="28"/>
+    </row>
+    <row r="24" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="29"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="35"/>
     </row>
     <row r="25" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
@@ -1257,19 +1297,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B5:G24">
-    <cfRule type="expression" dxfId="7" priority="4">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H5:H24">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1317,7 +1352,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E3" s="24" t="s">
         <v>28</v>
@@ -1329,173 +1364,203 @@
         <v>29</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="I3" s="24" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8"/>
       <c r="C5" s="2"/>
       <c r="D5" s="15"/>
       <c r="E5" s="15"/>
       <c r="F5" s="15"/>
       <c r="G5" s="2"/>
-      <c r="I5" s="26"/>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B6" s="8"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H5" s="26"/>
+      <c r="I5" s="28"/>
+    </row>
+    <row r="6" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="29"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="34"/>
+    </row>
+    <row r="7" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="8"/>
       <c r="C7" s="2"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B8" s="8"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H7" s="26"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="29"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="34"/>
+    </row>
+    <row r="9" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="8"/>
       <c r="C9" s="2"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B10" s="8"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H9" s="26"/>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="29"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="34"/>
+    </row>
+    <row r="11" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="8"/>
       <c r="C11" s="2"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B12" s="8"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H11" s="26"/>
+      <c r="I11" s="6"/>
+    </row>
+    <row r="12" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="29"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="34"/>
+    </row>
+    <row r="13" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="8"/>
       <c r="C13" s="2"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B14" s="8"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H13" s="26"/>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="29"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="34"/>
+    </row>
+    <row r="15" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="8"/>
       <c r="C15" s="2"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
-      <c r="I15" s="2"/>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B16" s="8"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H15" s="26"/>
+      <c r="I15" s="6"/>
+    </row>
+    <row r="16" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="29"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="34"/>
+    </row>
+    <row r="17" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="8"/>
       <c r="C17" s="2"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
-      <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B18" s="8"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H17" s="26"/>
+      <c r="I17" s="6"/>
+    </row>
+    <row r="18" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="34"/>
+    </row>
+    <row r="19" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="8"/>
       <c r="C19" s="2"/>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
-      <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B20" s="8"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H19" s="26"/>
+      <c r="I19" s="6"/>
+    </row>
+    <row r="20" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="29"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="34"/>
+    </row>
+    <row r="21" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="8"/>
       <c r="C21" s="2"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
-      <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="8"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="I22" s="2"/>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="H21" s="26"/>
+      <c r="I21" s="6"/>
+    </row>
+    <row r="22" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="29"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="34"/>
+    </row>
+    <row r="23" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="8"/>
       <c r="C23" s="2"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
-      <c r="I23" s="2"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B24" s="8"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="I24" s="2"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="6"/>
+    </row>
+    <row r="24" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="29"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="34"/>
     </row>
     <row r="25" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="9" t="s">
@@ -1543,11 +1608,6 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B5:H24">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>ISEVEN(ROW())</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="I5:I24">
     <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"C"</formula>

</xml_diff>

<commit_message>
Shorten buyerslist-infor rationale and preserve tier-total row heights
Tighten Rationale column guidance from ~150-350 chars to ~100-230 chars
(roughly 2/3 length) while keeping IB tone; rewrite the four strong
examples to the new length.

Add an explicit row-height reset in Step 7b: openpyxl's delete_rows
does not shift row_dimensions, so the three tier-total rows inherit
the 28.5pt height of the deleted buyer rows. Force them back to
14.25pt after deletion.

Also pull in the latest template (formatting tweaks) from the user's
Claude Access Folder.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Buyers List Template.xlsx
+++ b/infor-workflows/templates/INFOR Buyers List Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude Access Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66AD0C38-56CC-485A-ABB5-17C52B174AF8}"/>
+  <xr:revisionPtr revIDLastSave="373" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{532CED18-CB4C-4FC5-B47A-711485741B3D}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -277,7 +277,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -323,17 +323,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="hair">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -347,11 +375,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -361,12 +384,6 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -394,48 +411,86 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="6">
     <dxf>
       <font>
         <b/>
         <i val="0"/>
         <color rgb="FF00B050"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -443,11 +498,6 @@
         <i val="0"/>
         <color rgb="FFFFC000"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF3F6CC"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -455,11 +505,6 @@
         <i val="0"/>
         <color rgb="FFC00000"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -467,11 +512,6 @@
         <i val="0"/>
         <color rgb="FF00B050"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFCC"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -479,11 +519,6 @@
         <i val="0"/>
         <color rgb="FFFFC000"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF3F6CC"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -491,18 +526,6 @@
         <i val="0"/>
         <color rgb="FFC00000"/>
       </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -844,175 +867,175 @@
   <dimension ref="B1:F17"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="1" width="2.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="3" spans="2:6" ht="3" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
+      <c r="B4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
     </row>
     <row r="5" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
     </row>
     <row r="6" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
     </row>
     <row r="7" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
     </row>
     <row r="8" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="42"/>
+      <c r="F8" s="42"/>
     </row>
     <row r="9" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
     </row>
     <row r="10" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
     </row>
     <row r="11" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
     </row>
     <row r="12" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="4"/>
-      <c r="C13" s="5" t="s">
+      <c r="B13" s="3"/>
+      <c r="C13" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="12" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" spans="2:6" ht="3" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="13"/>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="11">
         <f>+'Strategic Buyers'!$H$25</f>
         <v>0</v>
       </c>
-      <c r="D15" s="17">
+      <c r="D15" s="11">
         <f>+'Strategic Buyers'!$H$26</f>
         <v>0</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="11">
         <f>+'Strategic Buyers'!$H$27</f>
         <v>0</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="14">
         <f>SUM(C15:E15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="11">
         <f>+'Financial Buyers'!$I$25</f>
         <v>0</v>
       </c>
-      <c r="D16" s="17">
+      <c r="D16" s="11">
         <f>+'Financial Buyers'!$I$26</f>
         <v>0</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="11">
         <f>+'Financial Buyers'!$I$27</f>
         <v>0</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="14">
         <f>SUM(C16:E16)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="16">
         <f>SUM(C15:C16)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="22">
+      <c r="D17" s="16">
         <f t="shared" ref="D17:F17" si="0">SUM(D15:D16)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F17" s="23">
+      <c r="F17" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1041,257 +1064,266 @@
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
     <col min="3" max="5" width="12.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="30.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="50.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="75.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" style="1" customWidth="1"/>
     <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="8"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="28"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23"/>
     </row>
     <row r="6" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="29"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="35"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="29"/>
     </row>
     <row r="7" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="8"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="16"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="28"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="35"/>
     </row>
     <row r="8" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="29"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="35"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="29"/>
     </row>
     <row r="9" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="8"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="16"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="28"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="35"/>
     </row>
     <row r="10" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="29"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="35"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="29"/>
     </row>
     <row r="11" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="8"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="16"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="28"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="35"/>
     </row>
     <row r="12" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="35"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="29"/>
     </row>
     <row r="13" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="8"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="16"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="28"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="35"/>
     </row>
     <row r="14" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="29"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="35"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="29"/>
     </row>
     <row r="15" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="8"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="16"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="28"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="35"/>
     </row>
     <row r="16" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="35"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="29"/>
     </row>
     <row r="17" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="8"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="16"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="28"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
     </row>
     <row r="18" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="35"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="29"/>
     </row>
     <row r="19" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="8"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="16"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="28"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="35"/>
     </row>
     <row r="20" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="29"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="33"/>
-      <c r="H20" s="35"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="29"/>
     </row>
     <row r="21" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="8"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="16"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="28"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="35"/>
     </row>
     <row r="22" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="29"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="35"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="29"/>
     </row>
     <row r="23" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="8"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="16"/>
-      <c r="G23" s="26"/>
-      <c r="H23" s="28"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="35"/>
     </row>
     <row r="24" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="29"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="35"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="41"/>
     </row>
     <row r="25" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="10">
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="8">
         <f>COUNTIF($H$5:$H$24,"A")</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="12">
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="8">
         <f>COUNTIF($H$5:$H$24,"B")</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="14">
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="10">
         <f>COUNTIF($H$5:$H$24,"C")</f>
         <v>0</v>
       </c>
@@ -1321,288 +1353,297 @@
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
     <col min="3" max="6" width="12.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="30.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="50.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="75.7109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="12.7109375" style="1" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="F2" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="24" t="s">
+      <c r="G2" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="24" t="s">
+      <c r="I3" s="18" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="8"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="28"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="23"/>
     </row>
     <row r="6" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="29"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="33"/>
-      <c r="I6" s="34"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="25"/>
     </row>
     <row r="7" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="8"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="6"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="31"/>
     </row>
     <row r="8" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="29"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="34"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="25"/>
     </row>
     <row r="9" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="8"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="6"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="31"/>
     </row>
     <row r="10" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="29"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="34"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="25"/>
     </row>
     <row r="11" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="8"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="6"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="31"/>
     </row>
     <row r="12" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="31"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="31"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="34"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="25"/>
     </row>
     <row r="13" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="8"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="6"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="31"/>
     </row>
     <row r="14" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="29"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="33"/>
-      <c r="I14" s="34"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="25"/>
     </row>
     <row r="15" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="8"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="6"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="31"/>
     </row>
     <row r="16" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="32"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="34"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="25"/>
     </row>
     <row r="17" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="8"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="6"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="31"/>
     </row>
     <row r="18" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="32"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="34"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="25"/>
     </row>
     <row r="19" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="8"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="6"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="31"/>
     </row>
     <row r="20" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="29"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="33"/>
-      <c r="I20" s="34"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="25"/>
     </row>
     <row r="21" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="8"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="6"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="31"/>
     </row>
     <row r="22" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="29"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="31"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="34"/>
+      <c r="B22" s="24"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="25"/>
     </row>
     <row r="23" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="8"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="H23" s="26"/>
-      <c r="I23" s="6"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="33"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="31"/>
     </row>
     <row r="24" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="29"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="34"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="37"/>
     </row>
     <row r="25" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="10">
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="8">
         <f>COUNTIF($I$5:$I$24,"A")</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="12">
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="8">
         <f>COUNTIF($I$5:$I$24,"B")</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="14">
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="10">
         <f>COUNTIF($I$5:$I$24,"C")</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Standardize M&A and Portfolio Companies column formats in buyerslist-infor
Replace free-form ≤30-char guidance with structured formats:

- Strategic Buyers · M&A activity (col F):
  "Target Name - YY, Target Name - YY, Target Name - YY" (max 3)
- Financial Buyers · Portfolio Companies (col G):
  "PortCo Name (Current), PortCo Name (Exited), ..." (max 3)

When more than 3 entries exist, prioritize by sector/thesis fit first,
then recency. YY is the 2-digit year of deal announcement.

Also fix a stale Rationale char-count (≈150-350) in the Financial
Buyers character-limits table that was missed in the previous PR; now
aligned with the ≈100-230 char guidance used everywhere else.

Pulls in the latest buyers list template with the user's formatting
tweaks.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Buyers List Template.xlsx
+++ b/infor-workflows/templates/INFOR Buyers List Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude Access Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="373" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{532CED18-CB4C-4FC5-B47A-711485741B3D}"/>
+  <xr:revisionPtr revIDLastSave="397" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70D34220-A1A5-432E-8B9D-E8CE1DACDA32}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -358,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -433,9 +433,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -451,9 +448,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -467,9 +461,6 @@
     </xf>
     <xf numFmtId="165" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -887,73 +878,73 @@
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
     </row>
     <row r="5" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
     </row>
     <row r="6" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
+      <c r="C6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="39"/>
     </row>
     <row r="7" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="42"/>
-      <c r="D7" s="42"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
     </row>
     <row r="8" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
     </row>
     <row r="9" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="42"/>
-      <c r="D9" s="42"/>
-      <c r="E9" s="42"/>
-      <c r="F9" s="42"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
     </row>
     <row r="10" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="42"/>
-      <c r="D10" s="42"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
     </row>
     <row r="12" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1120,171 +1111,171 @@
       <c r="C6" s="25"/>
       <c r="D6" s="25"/>
       <c r="E6" s="26"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="29"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="28"/>
     </row>
     <row r="7" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="30"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="35"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="33"/>
     </row>
     <row r="8" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="24"/>
       <c r="C8" s="25"/>
       <c r="D8" s="25"/>
       <c r="E8" s="26"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="28"/>
     </row>
     <row r="9" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="30"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="35"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="33"/>
     </row>
     <row r="10" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="24"/>
       <c r="C10" s="25"/>
       <c r="D10" s="25"/>
       <c r="E10" s="26"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="29"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="28"/>
     </row>
     <row r="11" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="33"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="35"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="33"/>
     </row>
     <row r="12" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="24"/>
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
       <c r="E12" s="26"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="29"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="28"/>
     </row>
     <row r="13" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="30"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="33"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="35"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="33"/>
     </row>
     <row r="14" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="24"/>
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="26"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="29"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="28"/>
     </row>
     <row r="15" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="30"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="35"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="33"/>
     </row>
     <row r="16" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="24"/>
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
       <c r="E16" s="26"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="29"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="28"/>
     </row>
     <row r="17" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="30"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="35"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="33"/>
     </row>
     <row r="18" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="24"/>
       <c r="C18" s="25"/>
       <c r="D18" s="25"/>
       <c r="E18" s="26"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="29"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="28"/>
     </row>
     <row r="19" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="30"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="35"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="33"/>
     </row>
     <row r="20" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="24"/>
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
       <c r="E20" s="26"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="29"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="21" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="30"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="35"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="33"/>
     </row>
     <row r="22" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="24"/>
       <c r="C22" s="25"/>
       <c r="D22" s="25"/>
       <c r="E22" s="26"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="29"/>
+      <c r="F22" s="25"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="28"/>
     </row>
     <row r="23" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="30"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="35"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="33"/>
     </row>
     <row r="24" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="41"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="38"/>
     </row>
     <row r="25" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="7" t="s">
@@ -1419,19 +1410,19 @@
       <c r="D6" s="26"/>
       <c r="E6" s="26"/>
       <c r="F6" s="26"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="28"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="27"/>
       <c r="I6" s="25"/>
     </row>
     <row r="7" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="30"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="31"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="30"/>
     </row>
     <row r="8" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="24"/>
@@ -1439,19 +1430,19 @@
       <c r="D8" s="26"/>
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="28"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="27"/>
       <c r="I8" s="25"/>
     </row>
     <row r="9" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="30"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="31"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="30"/>
     </row>
     <row r="10" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="24"/>
@@ -1459,19 +1450,19 @@
       <c r="D10" s="26"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="28"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="27"/>
       <c r="I10" s="25"/>
     </row>
     <row r="11" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="33"/>
-      <c r="H11" s="34"/>
-      <c r="I11" s="31"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="30"/>
     </row>
     <row r="12" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="24"/>
@@ -1479,19 +1470,19 @@
       <c r="D12" s="26"/>
       <c r="E12" s="26"/>
       <c r="F12" s="26"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="28"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="27"/>
       <c r="I12" s="25"/>
     </row>
     <row r="13" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="30"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="31"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="30"/>
     </row>
     <row r="14" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="24"/>
@@ -1499,19 +1490,19 @@
       <c r="D14" s="26"/>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="28"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="27"/>
       <c r="I14" s="25"/>
     </row>
     <row r="15" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="30"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="31"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="30"/>
     </row>
     <row r="16" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="24"/>
@@ -1519,19 +1510,19 @@
       <c r="D16" s="26"/>
       <c r="E16" s="26"/>
       <c r="F16" s="26"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="28"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="27"/>
       <c r="I16" s="25"/>
     </row>
     <row r="17" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="30"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="31"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="30"/>
     </row>
     <row r="18" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="24"/>
@@ -1539,19 +1530,19 @@
       <c r="D18" s="26"/>
       <c r="E18" s="26"/>
       <c r="F18" s="26"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="28"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="27"/>
       <c r="I18" s="25"/>
     </row>
     <row r="19" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="30"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="31"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="30"/>
     </row>
     <row r="20" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="24"/>
@@ -1559,19 +1550,19 @@
       <c r="D20" s="26"/>
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="28"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="27"/>
       <c r="I20" s="25"/>
     </row>
     <row r="21" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="30"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="31"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="30"/>
     </row>
     <row r="22" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="24"/>
@@ -1579,29 +1570,29 @@
       <c r="D22" s="26"/>
       <c r="E22" s="26"/>
       <c r="F22" s="26"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="28"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="27"/>
       <c r="I22" s="25"/>
     </row>
     <row r="23" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="30"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="32"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="33"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="31"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="30"/>
     </row>
     <row r="24" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="37"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="35"/>
     </row>
     <row r="25" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="7" t="s">

</xml_diff>

<commit_message>
Refresh INFOR Buyers List template with latest formatting tweaks
Pulls in the user's updated template. Sheet names, cell anchors, COUNTIF
total rows, and the 28.5pt / 14.25pt row-height pattern the skill relies
on are unchanged. Visible change: Vertical (Strategic · col D) and
Sector Focus (Financial · col F) column widths widened from 12.7 to
20.7 so those labels no longer truncate.

No skill code changes required.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Buyers List Template.xlsx
+++ b/infor-workflows/templates/INFOR Buyers List Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude Access Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="397" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70D34220-A1A5-432E-8B9D-E8CE1DACDA32}"/>
+  <xr:revisionPtr revIDLastSave="444" documentId="8_{A4A751D6-76C9-439E-98F6-E6A1D51A9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FB0C427-0507-4460-AC45-B02519A2A2CF}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B531B8E-4F5F-4F93-8808-1C6FD959FAAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -277,7 +277,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -343,22 +343,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="hair">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -453,23 +442,39 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -878,73 +883,73 @@
       <c r="B4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
     </row>
     <row r="5" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
     </row>
     <row r="6" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
     </row>
     <row r="7" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
     </row>
     <row r="8" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
     </row>
     <row r="9" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
     </row>
     <row r="10" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
     </row>
     <row r="11" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
     </row>
     <row r="12" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1053,7 +1058,9 @@
   <cols>
     <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
-    <col min="3" max="5" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="30.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="75.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" style="1" customWidth="1"/>
@@ -1102,7 +1109,7 @@
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="21"/>
-      <c r="F5" s="5"/>
+      <c r="F5" s="35"/>
       <c r="G5" s="22"/>
       <c r="H5" s="23"/>
     </row>
@@ -1111,7 +1118,7 @@
       <c r="C6" s="25"/>
       <c r="D6" s="25"/>
       <c r="E6" s="26"/>
-      <c r="F6" s="25"/>
+      <c r="F6" s="36"/>
       <c r="G6" s="27"/>
       <c r="H6" s="28"/>
     </row>
@@ -1120,7 +1127,7 @@
       <c r="C7" s="30"/>
       <c r="D7" s="30"/>
       <c r="E7" s="31"/>
-      <c r="F7" s="30"/>
+      <c r="F7" s="37"/>
       <c r="G7" s="32"/>
       <c r="H7" s="33"/>
     </row>
@@ -1129,7 +1136,7 @@
       <c r="C8" s="25"/>
       <c r="D8" s="25"/>
       <c r="E8" s="26"/>
-      <c r="F8" s="25"/>
+      <c r="F8" s="36"/>
       <c r="G8" s="27"/>
       <c r="H8" s="28"/>
     </row>
@@ -1138,7 +1145,7 @@
       <c r="C9" s="30"/>
       <c r="D9" s="30"/>
       <c r="E9" s="31"/>
-      <c r="F9" s="30"/>
+      <c r="F9" s="37"/>
       <c r="G9" s="32"/>
       <c r="H9" s="33"/>
     </row>
@@ -1147,7 +1154,7 @@
       <c r="C10" s="25"/>
       <c r="D10" s="25"/>
       <c r="E10" s="26"/>
-      <c r="F10" s="25"/>
+      <c r="F10" s="36"/>
       <c r="G10" s="27"/>
       <c r="H10" s="28"/>
     </row>
@@ -1156,7 +1163,7 @@
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
       <c r="E11" s="31"/>
-      <c r="F11" s="30"/>
+      <c r="F11" s="37"/>
       <c r="G11" s="32"/>
       <c r="H11" s="33"/>
     </row>
@@ -1165,7 +1172,7 @@
       <c r="C12" s="25"/>
       <c r="D12" s="25"/>
       <c r="E12" s="26"/>
-      <c r="F12" s="25"/>
+      <c r="F12" s="36"/>
       <c r="G12" s="27"/>
       <c r="H12" s="28"/>
     </row>
@@ -1174,7 +1181,7 @@
       <c r="C13" s="30"/>
       <c r="D13" s="30"/>
       <c r="E13" s="31"/>
-      <c r="F13" s="30"/>
+      <c r="F13" s="37"/>
       <c r="G13" s="32"/>
       <c r="H13" s="33"/>
     </row>
@@ -1183,7 +1190,7 @@
       <c r="C14" s="25"/>
       <c r="D14" s="25"/>
       <c r="E14" s="26"/>
-      <c r="F14" s="25"/>
+      <c r="F14" s="36"/>
       <c r="G14" s="27"/>
       <c r="H14" s="28"/>
     </row>
@@ -1192,7 +1199,7 @@
       <c r="C15" s="30"/>
       <c r="D15" s="30"/>
       <c r="E15" s="31"/>
-      <c r="F15" s="30"/>
+      <c r="F15" s="37"/>
       <c r="G15" s="32"/>
       <c r="H15" s="33"/>
     </row>
@@ -1201,7 +1208,7 @@
       <c r="C16" s="25"/>
       <c r="D16" s="25"/>
       <c r="E16" s="26"/>
-      <c r="F16" s="25"/>
+      <c r="F16" s="36"/>
       <c r="G16" s="27"/>
       <c r="H16" s="28"/>
     </row>
@@ -1210,7 +1217,7 @@
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
       <c r="E17" s="31"/>
-      <c r="F17" s="30"/>
+      <c r="F17" s="37"/>
       <c r="G17" s="32"/>
       <c r="H17" s="33"/>
     </row>
@@ -1219,7 +1226,7 @@
       <c r="C18" s="25"/>
       <c r="D18" s="25"/>
       <c r="E18" s="26"/>
-      <c r="F18" s="25"/>
+      <c r="F18" s="36"/>
       <c r="G18" s="27"/>
       <c r="H18" s="28"/>
     </row>
@@ -1228,7 +1235,7 @@
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
       <c r="E19" s="31"/>
-      <c r="F19" s="30"/>
+      <c r="F19" s="37"/>
       <c r="G19" s="32"/>
       <c r="H19" s="33"/>
     </row>
@@ -1237,7 +1244,7 @@
       <c r="C20" s="25"/>
       <c r="D20" s="25"/>
       <c r="E20" s="26"/>
-      <c r="F20" s="25"/>
+      <c r="F20" s="36"/>
       <c r="G20" s="27"/>
       <c r="H20" s="28"/>
     </row>
@@ -1246,7 +1253,7 @@
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
       <c r="E21" s="31"/>
-      <c r="F21" s="30"/>
+      <c r="F21" s="37"/>
       <c r="G21" s="32"/>
       <c r="H21" s="33"/>
     </row>
@@ -1255,7 +1262,7 @@
       <c r="C22" s="25"/>
       <c r="D22" s="25"/>
       <c r="E22" s="26"/>
-      <c r="F22" s="25"/>
+      <c r="F22" s="36"/>
       <c r="G22" s="27"/>
       <c r="H22" s="28"/>
     </row>
@@ -1264,29 +1271,29 @@
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
       <c r="E23" s="31"/>
-      <c r="F23" s="30"/>
+      <c r="F23" s="37"/>
       <c r="G23" s="32"/>
       <c r="H23" s="33"/>
     </row>
     <row r="24" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="34"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="43"/>
     </row>
     <row r="25" spans="2:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="8">
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="45">
         <f>COUNTIF($H$5:$H$24,"A")</f>
         <v>0</v>
       </c>
@@ -1342,7 +1349,8 @@
   <cols>
     <col min="1" max="1" width="2.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
-    <col min="3" max="6" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="5" width="12.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="30.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="75.7109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="12.7109375" style="1" customWidth="1"/>
@@ -1400,7 +1408,7 @@
       <c r="D5" s="21"/>
       <c r="E5" s="21"/>
       <c r="F5" s="21"/>
-      <c r="G5" s="5"/>
+      <c r="G5" s="35"/>
       <c r="H5" s="22"/>
       <c r="I5" s="23"/>
     </row>
@@ -1410,7 +1418,7 @@
       <c r="D6" s="26"/>
       <c r="E6" s="26"/>
       <c r="F6" s="26"/>
-      <c r="G6" s="25"/>
+      <c r="G6" s="36"/>
       <c r="H6" s="27"/>
       <c r="I6" s="25"/>
     </row>
@@ -1420,7 +1428,7 @@
       <c r="D7" s="31"/>
       <c r="E7" s="31"/>
       <c r="F7" s="31"/>
-      <c r="G7" s="30"/>
+      <c r="G7" s="37"/>
       <c r="H7" s="32"/>
       <c r="I7" s="30"/>
     </row>
@@ -1430,7 +1438,7 @@
       <c r="D8" s="26"/>
       <c r="E8" s="26"/>
       <c r="F8" s="26"/>
-      <c r="G8" s="25"/>
+      <c r="G8" s="36"/>
       <c r="H8" s="27"/>
       <c r="I8" s="25"/>
     </row>
@@ -1440,7 +1448,7 @@
       <c r="D9" s="31"/>
       <c r="E9" s="31"/>
       <c r="F9" s="31"/>
-      <c r="G9" s="30"/>
+      <c r="G9" s="37"/>
       <c r="H9" s="32"/>
       <c r="I9" s="30"/>
     </row>
@@ -1450,7 +1458,7 @@
       <c r="D10" s="26"/>
       <c r="E10" s="26"/>
       <c r="F10" s="26"/>
-      <c r="G10" s="25"/>
+      <c r="G10" s="36"/>
       <c r="H10" s="27"/>
       <c r="I10" s="25"/>
     </row>
@@ -1460,7 +1468,7 @@
       <c r="D11" s="31"/>
       <c r="E11" s="31"/>
       <c r="F11" s="31"/>
-      <c r="G11" s="30"/>
+      <c r="G11" s="37"/>
       <c r="H11" s="32"/>
       <c r="I11" s="30"/>
     </row>
@@ -1470,7 +1478,7 @@
       <c r="D12" s="26"/>
       <c r="E12" s="26"/>
       <c r="F12" s="26"/>
-      <c r="G12" s="25"/>
+      <c r="G12" s="36"/>
       <c r="H12" s="27"/>
       <c r="I12" s="25"/>
     </row>
@@ -1480,7 +1488,7 @@
       <c r="D13" s="31"/>
       <c r="E13" s="31"/>
       <c r="F13" s="31"/>
-      <c r="G13" s="30"/>
+      <c r="G13" s="37"/>
       <c r="H13" s="32"/>
       <c r="I13" s="30"/>
     </row>
@@ -1490,7 +1498,7 @@
       <c r="D14" s="26"/>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
-      <c r="G14" s="25"/>
+      <c r="G14" s="36"/>
       <c r="H14" s="27"/>
       <c r="I14" s="25"/>
     </row>
@@ -1500,7 +1508,7 @@
       <c r="D15" s="31"/>
       <c r="E15" s="31"/>
       <c r="F15" s="31"/>
-      <c r="G15" s="30"/>
+      <c r="G15" s="37"/>
       <c r="H15" s="32"/>
       <c r="I15" s="30"/>
     </row>
@@ -1510,7 +1518,7 @@
       <c r="D16" s="26"/>
       <c r="E16" s="26"/>
       <c r="F16" s="26"/>
-      <c r="G16" s="25"/>
+      <c r="G16" s="36"/>
       <c r="H16" s="27"/>
       <c r="I16" s="25"/>
     </row>
@@ -1520,7 +1528,7 @@
       <c r="D17" s="31"/>
       <c r="E17" s="31"/>
       <c r="F17" s="31"/>
-      <c r="G17" s="30"/>
+      <c r="G17" s="37"/>
       <c r="H17" s="32"/>
       <c r="I17" s="30"/>
     </row>
@@ -1530,7 +1538,7 @@
       <c r="D18" s="26"/>
       <c r="E18" s="26"/>
       <c r="F18" s="26"/>
-      <c r="G18" s="25"/>
+      <c r="G18" s="36"/>
       <c r="H18" s="27"/>
       <c r="I18" s="25"/>
     </row>
@@ -1540,7 +1548,7 @@
       <c r="D19" s="31"/>
       <c r="E19" s="31"/>
       <c r="F19" s="31"/>
-      <c r="G19" s="30"/>
+      <c r="G19" s="37"/>
       <c r="H19" s="32"/>
       <c r="I19" s="30"/>
     </row>
@@ -1550,7 +1558,7 @@
       <c r="D20" s="26"/>
       <c r="E20" s="26"/>
       <c r="F20" s="26"/>
-      <c r="G20" s="25"/>
+      <c r="G20" s="36"/>
       <c r="H20" s="27"/>
       <c r="I20" s="25"/>
     </row>
@@ -1560,7 +1568,7 @@
       <c r="D21" s="31"/>
       <c r="E21" s="31"/>
       <c r="F21" s="31"/>
-      <c r="G21" s="30"/>
+      <c r="G21" s="37"/>
       <c r="H21" s="32"/>
       <c r="I21" s="30"/>
     </row>
@@ -1570,7 +1578,7 @@
       <c r="D22" s="26"/>
       <c r="E22" s="26"/>
       <c r="F22" s="26"/>
-      <c r="G22" s="25"/>
+      <c r="G22" s="36"/>
       <c r="H22" s="27"/>
       <c r="I22" s="25"/>
     </row>
@@ -1580,31 +1588,31 @@
       <c r="D23" s="31"/>
       <c r="E23" s="31"/>
       <c r="F23" s="31"/>
-      <c r="G23" s="30"/>
+      <c r="G23" s="37"/>
       <c r="H23" s="32"/>
       <c r="I23" s="30"/>
     </row>
     <row r="24" spans="2:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="34"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="35"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="39"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="42"/>
+      <c r="I24" s="39"/>
     </row>
     <row r="25" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="8">
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="45">
         <f>COUNTIF($I$5:$I$24,"A")</f>
         <v>0</v>
       </c>

</xml_diff>